<commit_message>
feat: expand buqi effects and build catalog
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Buqi/BuqiEcho.xlsx
+++ b/Design/Excel/GameHot/Datas/Buqi/BuqiEcho.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>急令试影</t>
+          <t>攻击试影</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>冲刺试影</t>
+          <t>冲锋试影</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>echo-fast-early;fast;100;0;0;efe-board,W8-005,Improved,0,None|efe-urgent,W8-003,Normal,2,None|efe-buffer,W8-007,Normal,3,None</t>
+          <t>echo-fast-early;fast;100;0;0;efe-board,W8-005,Improved,0,None|efe-urgent,W8-003,Normal,2,None|efe-shield,W8-007,Normal,3,None</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>护体试影</t>
+          <t>护盾试影</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>echo-buffer-lesson;buffer;100;0;0;ebl-buffer,W8-007,Normal,0,None|ebl-risk,W8-008,Normal,1,A-04|ebl-center,W8-012,Normal,2,None</t>
+          <t>echo-buffer-lesson;buffer;100;0;0;ebl-shield,W8-007,Normal,0,None|ebl-list,W8-008,Normal,1,A-04|ebl-core,W8-012,Normal,2,None</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>灾备试影</t>
+          <t>堡垒试影</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>echo-buffer-early;buffer;100;0;0;ebe-center,W8-012,Normal,0,None|ebe-buffer,W8-007,Improved,3,None</t>
+          <t>echo-buffer-early;buffer;100;0;0;ebe-core,W8-012,Normal,0,None|ebe-shield,W8-007,Improved,3,None</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>交接试影</t>
+          <t>连锁试影</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>echo-chain-lesson;chain;100;0;0;ecl-hand,W8-013,Normal,0,None|ecl-sign,W8-014,Normal,1,A-03|ecl-node,W8-015,Normal,2,None</t>
+          <t>echo-chain-lesson;chain;100;0;0;ecl-wire,W8-013,Normal,0,None|ecl-mark,W8-014,Normal,1,A-03|ecl-node,W8-015,Normal,2,None</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>联签试影</t>
+          <t>充能试影</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -678,7 +678,277 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>echo-chain-early;chain;100;0;0;ece-hand,W8-013,Improved,0,None|ece-sign,W8-014,Normal,1,None|ece-node,W8-015,Normal,2,None</t>
+          <t>echo-chain-early;chain;100;0;0;ece-wire,W8-013,Improved,0,None|ece-mark,W8-014,Normal,1,None|ece-node,W8-015,Normal,2,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>echo-heal-lesson</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>治疗试影</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>lesson</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>echo-heal-lesson;heal;100;0;0;ehl-pack,W8-016,Normal,0,None|ehl-spring,W8-017,Normal,1,None|ehl-flag,W8-018,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>echo-heal-early</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>回春试影</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>echo-heal-early;heal;100;0;0;ehe-pack,W8-016,Improved,0,None|ehe-spring,W8-017,Normal,1,None|ehe-shield,W8-007,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>echo-poison-lesson</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>中毒试影</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>lesson</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>poison</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>echo-poison-lesson;poison;100;0;0;epl-needle,W8-019,Normal,0,None|epl-bottle,W8-020,Normal,1,None|epl-fog,W8-021,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>echo-poison-early</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>腐蚀试影</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>poison</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>echo-poison-early;poison;100;0;0;epe-needle,W8-019,Improved,0,None|epe-bottle,W8-020,Normal,1,None|epe-mirror,W8-025,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>echo-burn-lesson</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>灼烧试影</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>lesson</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>burn</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>echo-burn-lesson;burn;100;0;0;eburn-spark,W8-022,Normal,0,None|eburn-furnace,W8-023,Normal,1,None|eburn-array,W8-024,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>echo-burn-early</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>烈焰试影</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>burn</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>echo-burn-early;burn;100;0;0;ebe-spark,W8-022,Improved,0,None|ebe-furnace,W8-023,Normal,1,None|ebe-urgent,W8-003,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>echo-freeze-lesson</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>冰冻试影</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>lesson</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>freeze</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>echo-freeze-lesson;freeze;100;0;0;efz-mirror,W8-025,Normal,0,None|efz-lock,W8-026,Normal,1,None|efz-tower,W8-027,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>echo-freeze-early</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>霜锁试影</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>freeze</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>echo-freeze-early;freeze;100;0;0;efe-mirror,W8-025,Improved,0,None|efe-lock,W8-026,Normal,1,None|efe-shield,W8-007,Normal,3,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>echo-overload-lesson</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>过载试影</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>lesson</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>overload</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>echo-overload-lesson;overload;100;0;0;eol-battery,W8-028,Normal,0,None|eol-core,W8-030,Normal,1,None|eol-vent,W8-029,Normal,3,None|eol-board,W8-005,Normal,4,None</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>echo-overload-early</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>泄压试影</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>early</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>overload</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>echo-overload-early;overload;100;0;0;eoe-battery,W8-028,Improved,0,None|eoe-vent,W8-029,Normal,1,None|eoe-core,W8-030,Normal,2,None</t>
         </is>
       </c>
     </row>

</xml_diff>